<commit_message>
Actualización automática de noticias
</commit_message>
<xml_diff>
--- a/Data/Lambayeque/noticias_lambayeque_20260914_20260921.xlsx
+++ b/Data/Lambayeque/noticias_lambayeque_20260914_20260921.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,93 +537,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Visita del papa León XIV: 100,000 devotos asistirán a misa que se celebrará en Santa Cruz</t>
+          <t>Papa León XIV en Perú: ¿Qué días visitará Chiclayo, Cusco y Pucallpa?</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
-        <is>
-          <t>El alcalde de Santa Cruz, José Alarcón Dávila, quien actualmente se encuentra de licencia, declaró a la Agencia Andina que la visita del papa León XIV constituye una bendición para su provincia y un acontecimiento histórico, al tratarse del máximo representante de la Iglesia católica en el mundo.
-La población se encuentra conmovida por su fe religiosa y el deseo de reencontrarse con el sumo pontífice, quien recorrió diversos distritos de esta provincia durante su labor pastoral como obispo de Chiclayo, sostuvo el burgomaestre, al recordar que Robert Francis Prevost presidía las celebraciones religiosas en honor al Señor del Costado, patrón de Santa Cruz.
-“Somos una pequeña provincia de la región Cajamarca, pero con una inquebrantable fe religiosa que, con la visita del Papa, estará en los ojos del mundo.
-Él siempre visitó Santa Cruz durante su labor pastoral como obispo de Chiclayo y, en gratitud, nos estamos preparando para recibirlo de la mejor manera.
-Será un acontecimiento inolvidable”, precisó.
-Alarcón comentó que una comisión encargada de organizar la llegada del santo padre, integrada por representantes de la parroquia, la Municipalidad Provincial de Santa Cruz y el Gobierno Regional de Cajamarca, viene trabajando en el acondicionamiento del campo de aviación, donde se celebrará la misa el sábado 14 de noviembre, a las 10:00 horas.
-En otro momento, la autoridad municipal expresó su preocupación por la cantidad de personas que arribarán a su provincia.
-“Se está capacitando a los vecinos para que acondicionen sus viviendas y puedan alojar a los visitantes.
-La Dirección Regional de Comercio Exterior y Turismo de Cajamarca también viene capacitando a los propietarios de restaurantes y a los transportistas.
-Se espera recibir a unos 100,000 peregrinos”, afirmó.
-La provincia de Santa Cruz cuenta con más de 35,000 habitantes y está conformada por 11 distritos: Andabamba, Catache, Chancaybaños, La Esperanza, Ninabamba, Pulán, Saucepampa, Sexi, Uticyacu, Yauyucán y Santa Cruz.
-Sus principales actividades económicas son la agricultura y la ganadería, y mantiene una importante conexión comercial con la región Lambayeque.
-El burgomaestre señaló que su provincia es una de las más olvidadas de Cajamarca y espera que, con motivo de la visita del Papa, las autoridades regionales y nacionales atiendan sus principales necesidades.
-“Esperamos que el Papa pueda interceder ante la presidenta de la República para que se haga realidad el asfaltado de la carretera Santa Cruz-Chiclayo”, precisó.
-Atractivos turísticos Santa Cruz, conocida como la “Tierra de la Cordialidad”, posee innumerables atractivos turísticos, entre ellos el complejo de aguas termomedicinales de Chancaybaños, el puente colgante, la Laguna del Amor, las grutas de Ushcupishgo, las cataratas de Pulán y el bosque paleontológico de Piedra Chamana.
-Asimismo, destacan el Santuario de la Virgen de los Remedios, las ruinas de Poro Poro, el cerro Cotorumi, considerado un mirador natural de Santa Cruz; la catarata Pacchac y el área natural protegida Bosques Nublados de Udima, entre otros atractivos.
-En entrevista con la Agencia Andina, el profesor Yoni Ramos García, expresó que su provincia ha sido bendecida con la visita de Robert Francis Prevost y que aprovecharán esta oportunidad para mostrar a los visitantes sus principales atractivos turísticos.
-El anhelo de Santa Cruz es contar con un museo arqueológico donde se puedan exhibir piezas de cerámica, momias y otros restos históricos que actualmente se encuentran en la Dirección Desconcentrada de Cultura de Lambayeque.
-“Iniciamos las gestiones para que nos devuelvan estas piezas, pero no fue posible porque no contamos con un espacio adecuado para su conservación y exhibición”, precisó.
-“Creemos que Santa Cruz es una provincia bendecida por haber sido considerada por la máxima autoridad de la Iglesia católica.
-Agradecemos al papa León XIV por elegir nuestra provincia como parte de su visita al Perú.
-Estamos ante los ojos del mundo y esperamos que las autoridades consideren a Santa Cruz para que salga del olvido y reciba el apoyo que merece”, expresó el docente.
-Recorrido del Papa Durante el periodo en que Robert Francis Prevost fue obispo de la Diócesis de Chiclayo, a la que pertenece la provincia cajamarquina de Santa Cruz, recorrió los distritos de Chancaybaños, Yauyucán, Andabamba, Pulán, Catache y Santa Cruz, donde celebró misas con motivo de sus festividades patronales, dedicadas al Señor del Costado y a la Santísima Virgen de los Remedios de Litcán.
-Como obispo, también realizó bautizos y confirmaciones, recordó Yoni Ramos, quien precisó que la provincia de Santa Cruz cuenta con tres vías de acceso.
-Una de ellas es la ruta Chiclayo-Cumbil-Santa Cruz, con un recorrido aproximado de cuatro horas; y otra es la ruta Cajamarca-El Empalme-Catilluc-Tongod-Santa Cruz, que demanda un tiempo similar.
-La ruta más larga es Cajamarca-Hualgayoc-Chota-Lajas-Santa Cruz, cuyo recorrido demanda aproximadamente cinco horas.
-“También hay rutas de acceso para quienes vienen de las provincias de Jaén y Cutervo, por la zona de Cochabamba y Tambillo”, puntualizó.
-Más en Andina:</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://andina.pe/agencia/noticia-visita-del-papa-leon-xiv-100000-devotos-asistiran-a-misa-se-celebrara-santa-cruz-1092605.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Andina</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>46286</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Perú se prepara para recibir con júbilo al papa León XIV</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>La llegada del Sumo Pontífice es motivo de inmensa alegría para el pueblo peruano, que lo espera con anhelo pues representa el testimonio de especial afecto y cercanía espiritual que el Santo Padre guarda por el Perú, país que también es el suyo.
-El Vaticano anuncia programa oficial de visita de papa León XIV al Perú https://t.co/pVggQUuuib pic.twitter.com/byjGAxnCSs — Agencia Andina (@Agencia_Andina) September 21, 2026 El itinerario oficial incluye las ciudades de Lima, Chiclayo (Lambayeque), Santa Cruz de Succhabamba (Cajamarca), Pucallpa (Ucayali) y Cusco ; y, traza un peregrinaje por la diversidad geográfica, cultural y social del Perú.
-Asimismo, incluye lugares de especial significado para el Santo Padre, donde podrá conectar con el pueblo peruano de la Costa, la Sierra y la Selva de nuestro país, llevando un mensaje de paz, diálogo y reconciliación.
-???????? El Gobierno del Perú recibe con inmenso júbilo y emoción el anuncio oficial de la Santa Sede del programa de la Visita Apostólica de Su Santidad el Papa León XIV, que se llevará a cabo del 11 al 16 de noviembre.
-La tan anhelada llegada del Santo Padre al Perú, testimonio… — Presidencia del Perú ???? (@presidenciaperu) September 21, 2026 Programa oficial de visita de León XIV al Perú: el país espera con júbilo y esperanza la llegada del papa peruano El Perú entero abre sus brazos para recibir al Santo Padre en un encuentro que quedará grabado para siempre en la memoria y el corazón de nuestra nación.
-Más en Andina ???? El papa León XIV se dirige a la multitud desde la ventana del palacio apostólico con vistas a la Plaza de San Pedro durante el rezo del Ángelus dominical en el Vaticano, el 20 de septiembre de 2026.
-https://t.co/FGz2ph5Oro Foto de Andreas SOLARO / AFP pic.twitter.com/NZjYCuglSq — Agencia Andina (@Agencia_Andina) September 20, 2026</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://andina.pe/agencia/noticia-peru-se-prepara-para-recibir-jubilo-al-papa-leon-xiv-1092593.aspx</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Andina</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>46286</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Papa León XIV en Perú: ¿Qué días visitará Chiclayo, Cusco y Pucallpa?</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
         <is>
           <t>La programación, prevista del viernes 13 al domingo 15 de noviembre de 2026, contempla desplazamientos por Chiclayo, Pimentel, Santa Cruz de Succhabamba, Zaña, Cusco y Pucallpa, antes del retorno del Santo Padre a Lima.
 Viernes 13: inicio de actividades en Chiclayo La gira en provincias se iniciará en Chiclayo, la ciudad que tiene un fuerte vínculo con León XIV donde el Papa se desempeño como obispo de la Diócesis de Chiclayo desde 2015 al 2023.
@@ -661,16 +578,93 @@
 Más en Andina: Fenómeno El Niño: Kuélap refuerza acciones preventivas ante inicio de temporada de lluvias https://t.co/JMtz8ryIDC a través de @Agencia_Andina — Moisés Aylas Ortiz (@regionalesand) September 21, 2026</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-papa-leon-xiv-peru-dias-visitara-chiclayo-cusco-y-pucallpa-1092590.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Visita del papa León XIV: 100,000 devotos asistirán a misa que se celebrará en Santa Cruz</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>El alcalde de Santa Cruz, José Alarcón Dávila, quien actualmente se encuentra de licencia, declaró a la Agencia Andina que la visita del papa León XIV constituye una bendición para su provincia y un acontecimiento histórico, al tratarse del máximo representante de la Iglesia católica en el mundo.
+La población se encuentra conmovida por su fe religiosa y el deseo de reencontrarse con el sumo pontífice, quien recorrió diversos distritos de esta provincia durante su labor pastoral como obispo de Chiclayo, sostuvo el burgomaestre, al recordar que Robert Francis Prevost presidía las celebraciones religiosas en honor al Señor del Costado, patrón de Santa Cruz.
+“Somos una pequeña provincia de la región Cajamarca, pero con una inquebrantable fe religiosa que, con la visita del Papa, estará en los ojos del mundo.
+Él siempre visitó Santa Cruz durante su labor pastoral como obispo de Chiclayo y, en gratitud, nos estamos preparando para recibirlo de la mejor manera.
+Será un acontecimiento inolvidable”, precisó.
+Alarcón comentó que una comisión encargada de organizar la llegada del santo padre, integrada por representantes de la parroquia, la Municipalidad Provincial de Santa Cruz y el Gobierno Regional de Cajamarca, viene trabajando en el acondicionamiento del campo de aviación, donde se celebrará la misa el sábado 14 de noviembre, a las 10:00 horas.
+En otro momento, la autoridad municipal expresó su preocupación por la cantidad de personas que arribarán a su provincia.
+“Se está capacitando a los vecinos para que acondicionen sus viviendas y puedan alojar a los visitantes.
+La Dirección Regional de Comercio Exterior y Turismo de Cajamarca también viene capacitando a los propietarios de restaurantes y a los transportistas.
+Se espera recibir a unos 100,000 peregrinos”, afirmó.
+La provincia de Santa Cruz cuenta con más de 35,000 habitantes y está conformada por 11 distritos: Andabamba, Catache, Chancaybaños, La Esperanza, Ninabamba, Pulán, Saucepampa, Sexi, Uticyacu, Yauyucán y Santa Cruz.
+Sus principales actividades económicas son la agricultura y la ganadería, y mantiene una importante conexión comercial con la región Lambayeque.
+El burgomaestre señaló que su provincia es una de las más olvidadas de Cajamarca y espera que, con motivo de la visita del Papa, las autoridades regionales y nacionales atiendan sus principales necesidades.
+“Esperamos que el Papa pueda interceder ante la presidenta de la República para que se haga realidad el asfaltado de la carretera Santa Cruz-Chiclayo”, precisó.
+Atractivos turísticos Santa Cruz, conocida como la “Tierra de la Cordialidad”, posee innumerables atractivos turísticos, entre ellos el complejo de aguas termomedicinales de Chancaybaños, el puente colgante, la Laguna del Amor, las grutas de Ushcupishgo, las cataratas de Pulán y el bosque paleontológico de Piedra Chamana.
+Asimismo, destacan el Santuario de la Virgen de los Remedios, las ruinas de Poro Poro, el cerro Cotorumi, considerado un mirador natural de Santa Cruz; la catarata Pacchac y el área natural protegida Bosques Nublados de Udima, entre otros atractivos.
+En entrevista con la Agencia Andina, el profesor Yoni Ramos García, expresó que su provincia ha sido bendecida con la visita de Robert Francis Prevost y que aprovecharán esta oportunidad para mostrar a los visitantes sus principales atractivos turísticos.
+El anhelo de Santa Cruz es contar con un museo arqueológico donde se puedan exhibir piezas de cerámica, momias y otros restos históricos que actualmente se encuentran en la Dirección Desconcentrada de Cultura de Lambayeque.
+“Iniciamos las gestiones para que nos devuelvan estas piezas, pero no fue posible porque no contamos con un espacio adecuado para su conservación y exhibición”, precisó.
+“Creemos que Santa Cruz es una provincia bendecida por haber sido considerada por la máxima autoridad de la Iglesia católica.
+Agradecemos al papa León XIV por elegir nuestra provincia como parte de su visita al Perú.
+Estamos ante los ojos del mundo y esperamos que las autoridades consideren a Santa Cruz para que salga del olvido y reciba el apoyo que merece”, expresó el docente.
+Recorrido del Papa Durante el periodo en que Robert Francis Prevost fue obispo de la Diócesis de Chiclayo, a la que pertenece la provincia cajamarquina de Santa Cruz, recorrió los distritos de Chancaybaños, Yauyucán, Andabamba, Pulán, Catache y Santa Cruz, donde celebró misas con motivo de sus festividades patronales, dedicadas al Señor del Costado y a la Santísima Virgen de los Remedios de Litcán.
+Como obispo, también realizó bautizos y confirmaciones, recordó Yoni Ramos, quien precisó que la provincia de Santa Cruz cuenta con tres vías de acceso.
+Una de ellas es la ruta Chiclayo-Cumbil-Santa Cruz, con un recorrido aproximado de cuatro horas; y otra es la ruta Cajamarca-El Empalme-Catilluc-Tongod-Santa Cruz, que demanda un tiempo similar.
+La ruta más larga es Cajamarca-Hualgayoc-Chota-Lajas-Santa Cruz, cuyo recorrido demanda aproximadamente cinco horas.
+“También hay rutas de acceso para quienes vienen de las provincias de Jaén y Cutervo, por la zona de Cochabamba y Tambillo”, puntualizó.
+Más en Andina:</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-visita-del-papa-leon-xiv-100000-devotos-asistiran-a-misa-se-celebrara-santa-cruz-1092605.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gestión</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Faraón no se queda en el arroz y prepara su salto a tres nuevas categorías</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>El peruano tiene una característica que lo distingue de otros consumidores de la región: su afición por el arroz. De acuerdo con datos del INEI, el consumo de arroz en Perú se mantiene en niveles elevados, con 74 kg per cápita al año en 2026. En este mercado, uno de los principales actores es Productos Faraón, la segunda marca individual de arroz más grande del país, solo superada por el portafolio de Costeño Alimentos (grupo Camil). En un mercado de alto consumo, ¿cuáles son los planes de Faraón para seguir creciendo y, al mismo tiempo, diversificar su portafolio más allá del arroz? Tomás Padilla, CEO de Productos Faraón, señaló a Gestión que en el primer semestre de 2026 la compañía registró un crecimiento promedio de 8% en sus ventas, en línea con la evolución positiva que la marca ha mostrado en los últimos años. “Hay años que hemos tenido un crecimiento de 10%, otros de 15%. En esta primera mitad del año estamos creciendo a tasas de un dígito”, comentó. Uno de los factores detrás de este resultado es la preferencia del consumidor por las características del producto y la consistencia de su calidad. “La preferencia es principalmente por el consumidor que le sigue gustando la promesa que tiene la marca, que es un arroz que se granea, tampoco se masacotea, que sirve para recalentar, da buen rendimiento y sabor”, sostuvo. Esta propuesta, explicó, se ha construido a lo largo de los más de 20 años que lleva la marca en el mercado y se sustenta en un proceso que busca mantener un estándar de calidad desde el campo hasta la planta. En esta última, la compañía recibe el arroz con cáscara proveniente de agricultores locales y desarrolla las distintas etapas de procesamiento, que incluyen el secado industrial para reducir la humedad del grano, el descascarado, blanqueo y pulido, así como la clasificación por tamaño y la selección láser para retirar los granos defectuosos. “Por último, el arroz es empacado en distintas presentaciones comerciales”, contó. Para ello, la compañía trabaja con agricultores en un contexto marcado por el minifundio, donde las extensiones de cultivo pueden ser de una, cinco o 20 hectáreas. Esta característica implica organizar el trabajo de acuerdo con las distintas variedades de arroz, debido a que cada una tiene un comportamiento diferente durante la preparación. A esta preferencia se suma, según el ejecutivo, una mayor apuesta por el arroz nacional frente al importado. Este comportamiento de la demanda acompaña la expansión geográfica de Productos Faraón, que mantiene una presencia consolidada en Lima y ha avanzado hacia otras ciudades. Actualmente, la compañía está presente en Arequipa, Tacna y Cusco, así como en Piura, Chiclayo, Chimbote y Trujillo. En cuanto a los canales, el mercado tradicional continúa siendo un espacio central para la compañía. “Hace más o menos 15 años que entramos a los supermercados”, comentó. Actualmente, ambos canales tienen una participación similar en las ventas de la compañía, con una distribución que fluctúa alrededor del 50% para cada uno. “No nos centramos en un solo mercado”, arguyó. Paralelamente y como parte de su estrategia de crecimiento, Productos Faraón viene ampliando su portafolio de arroz en función de las nuevas necesidades y preferencias del consumidor. “Por ejemplo, tenemos arroces para chifas, arroces para menús, arroces gourmet, entre otros. Estamos en el proceso de diversificar nuestro producto estrella para llegar a todo tipo de consumidores”, expresó el CEO. Esta diversificación también apunta a la categoría de productos saludables. En detalle, la empresa ya comercializa arroz integral, vinculada a la tendencia de una alimentación con mayor contenido de fibra. Con respecto al corto plazo, Faraón prepara nuevas presentaciones y formatos más pequeños, con el objetivo de ampliar el consumo de arroz embolsado. Actualmente, la mayor parte del consumo en el país todavía se realiza a granel. “El Perú consume mayormente a granel, estaría en los más del 80%”, indicó. Frente a ello, la compañía busca avanzar hacia formatos que permitan una mejor conservación del producto y preserven sus condiciones de calidad e inocuidad. “Presentaciones más pequeñas y, sobre todo, que conserven mejor el producto, que no tenga contaminaciones, así puede durar mucho más en el tiempo y se preserva, sobre todo, la calidad del grano”, explicó. La apuesta contempla formatos de 500 gramos, 750 gramos y cinco kilos, con un mayor énfasis en presentaciones de hasta 10 kilos. Actualmente, el arroz embolsado en formatos pequeños representa alrededor del 25% de las ventas de la compañía. La nueva etapa también contempla una inversión en tecnología para el proceso y empaque. ¿Cuándo estarán en el mercado estas innovaciones? Padilla adelantó que estas nuevas presentaciones llegarían al mercado hacia finales de año. “Ya tenemos instalada nuestra planta de proceso”, comentó. Para este desarrollo, la empresa está destinando alrededor de US$ 1.5 millones, inversión que estará enfocada en la incorporación de nueva tecnología. “Estamos invirtiendo en tecnología para llevar al mercado un arroz con mejor fibra y mejores componentes, además de desarrollar presentaciones más pequeñas”, manifestó. La diversificación de Productos Faraón no se limita al arroz. La compañía también participa en la categoría de menestras, donde comercializa lentejas, pallares, garbanzos, arvejas y distintas variedades de frijoles. “Trabajamos tanto con productos nacionales como importados”, alegó. En esta categoría, la compañía también prepara nuevas presentaciones, con una apuesta por formatos pequeños, que estarían disponibles hacia finales de este año. La estrategia de diversificación también contempla ampliar el portafolio de Faraón hacia otras categorías de alimentos de consumo masivo. Entre las categorías que la compañía analiza se encuentran las harinas especiales, como la harina de arroz, además de pastas y aceites, aunque estas incorporaciones todavía se encuentran en proceso de evaluación. El ingreso a estas nuevas categorías está previsto para 2027, con una expectativa de lanzamiento durante el primer semestre de ese año. “La decisión responde a la búsqueda de nuevas oportunidades dentro del consumo masivo y a la demanda de los consumidores, por lo que siempre estamos buscando alternativas de negocios de consumo masivo”, anotó. Una de las principales preocupaciones para la empresa está relacionada con el impacto de Fenómeno El Niño en la producción de los agricultores que la abastecen. En Lambayeque, en particular, Padilla señaló que uno de los principales riesgos asociados a este evento climático es la aparición de plagas como la sogata y la hoja blanca. Ante a este escenario, la empresa viene tomando previsiones para asegurar el abastecimiento y atender la demanda. “Sí estamos previniendo y, en caso de los volúmenes, estamos tratando de tener más producto en stock para sostener la demanda de nuestro mercado”, adelantó. La compañía trabaja con una red de más de 1,000 agricultores y se abastece de distintas zonas de la costa y la selva. Entre ellas se encuentran Lambayeque, Sullana y Piura, además de Tumbes y el valle de Jequetepeque. También obtiene parte de su materia prima de Jaén y Bagua, así como de Nueva Cajamarca, en el Alto Mayo. “Hemos hecho un trabajo interesante con ellos, campaña a campaña, que nos apoyamos mutuamente”, anotó. Esta relación también permite a la empresa anticiparse a eventuales dificultades en la producción. “Si les va mal a ellos, también a nosotros nos va mal”, sostuvo. Actualmente, Productos Faraón concentra su infraestructura industrial en el norte: específicamente su planta está ubicada en Lambayeque (cerca a Chiclayo) y cuenta con un área total de aproximadamente 300,000 metros cuadrados (m2) destinada, entre otros usos, al almacenamiento de arroz. De este espacio, alrededor de 80,000 m2 corresponden al área industrial. La compañía, además, prepara la puesta en operación de una nueva planta en la selva, que complementará las operaciones del norte. “La nueva planta estará en funcionando el próximo año, posiblemente a fines de año”, reveló Padilla. La nueva infraestructura funcionará de manera independiente a la planta del norte y tendrá como uno de sus objetivos acercar a la compañía a los agricultores de esa zona. “Va a complementar la planta del norte, pero independiente, para estar más cerca del agricultor”, expresó. Con esta ampliación, Faraón prevé contar con dos plantas operativas hacia finales de 2027. El ejecutivo precisó que todavía no cuentan con el monto de inversión definido para la nueva planta, que incorporará nueva tecnología.</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://andina.pe/agencia/noticia-papa-leon-xiv-peru-dias-visitara-chiclayo-cusco-y-pucallpa-1092590.aspx</t>
+          <t>https://gestion.pe/economia/empresas/productos-faraon-ventas-crecen-8-y-prepara-nueva-planta-en-la-selva-para-2027-noticia/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Gestión</t>
+          <t>Andina</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -678,17 +672,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Faraón no se queda en el arroz y prepara su salto a tres nuevas categorías</t>
+          <t>Perú se prepara para recibir con júbilo al papa León XIV</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>El peruano tiene una característica que lo distingue de otros consumidores de la región: su afición por el arroz. De acuerdo con datos del INEI, el consumo de arroz en Perú se mantiene en niveles elevados, con 74 kg per cápita al año en 2026. En este mercado, uno de los principales actores es Productos Faraón, la segunda marca individual de arroz más grande del país, solo superada por el portafolio de Costeño Alimentos (grupo Camil). En un mercado de alto consumo, ¿cuáles son los planes de Faraón para seguir creciendo y, al mismo tiempo, diversificar su portafolio más allá del arroz? Tomás Padilla, CEO de Productos Faraón, señaló a Gestión que en el primer semestre de 2026 la compañía registró un crecimiento promedio de 8% en sus ventas, en línea con la evolución positiva que la marca ha mostrado en los últimos años. “Hay años que hemos tenido un crecimiento de 10%, otros de 15%. En esta primera mitad del año estamos creciendo a tasas de un dígito”, comentó. Uno de los factores detrás de este resultado es la preferencia del consumidor por las características del producto y la consistencia de su calidad. “La preferencia es principalmente por el consumidor que le sigue gustando la promesa que tiene la marca, que es un arroz que se granea, tampoco se masacotea, que sirve para recalentar, da buen rendimiento y sabor”, sostuvo. Esta propuesta, explicó, se ha construido a lo largo de los más de 20 años que lleva la marca en el mercado y se sustenta en un proceso que busca mantener un estándar de calidad desde el campo hasta la planta. En esta última, la compañía recibe el arroz con cáscara proveniente de agricultores locales y desarrolla las distintas etapas de procesamiento, que incluyen el secado industrial para reducir la humedad del grano, el descascarado, blanqueo y pulido, así como la clasificación por tamaño y la selección láser para retirar los granos defectuosos. “Por último, el arroz es empacado en distintas presentaciones comerciales”, contó. Para ello, la compañía trabaja con agricultores en un contexto marcado por el minifundio, donde las extensiones de cultivo pueden ser de una, cinco o 20 hectáreas. Esta característica implica organizar el trabajo de acuerdo con las distintas variedades de arroz, debido a que cada una tiene un comportamiento diferente durante la preparación. A esta preferencia se suma, según el ejecutivo, una mayor apuesta por el arroz nacional frente al importado. Este comportamiento de la demanda acompaña la expansión geográfica de Productos Faraón, que mantiene una presencia consolidada en Lima y ha avanzado hacia otras ciudades. Actualmente, la compañía está presente en Arequipa, Tacna y Cusco, así como en Piura, Chiclayo, Chimbote y Trujillo. En cuanto a los canales, el mercado tradicional continúa siendo un espacio central para la compañía. “Hace más o menos 15 años que entramos a los supermercados”, comentó. Actualmente, ambos canales tienen una participación similar en las ventas de la compañía, con una distribución que fluctúa alrededor del 50% para cada uno. “No nos centramos en un solo mercado”, arguyó. Paralelamente y como parte de su estrategia de crecimiento, Productos Faraón viene ampliando su portafolio de arroz en función de las nuevas necesidades y preferencias del consumidor. “Por ejemplo, tenemos arroces para chifas, arroces para menús, arroces gourmet, entre otros. Estamos en el proceso de diversificar nuestro producto estrella para llegar a todo tipo de consumidores”, expresó el CEO. Esta diversificación también apunta a la categoría de productos saludables. En detalle, la empresa ya comercializa arroz integral, vinculada a la tendencia de una alimentación con mayor contenido de fibra. Con respecto al corto plazo, Faraón prepara nuevas presentaciones y formatos más pequeños, con el objetivo de ampliar el consumo de arroz embolsado. Actualmente, la mayor parte del consumo en el país todavía se realiza a granel. “El Perú consume mayormente a granel, estaría en los más del 80%”, indicó. Frente a ello, la compañía busca avanzar hacia formatos que permitan una mejor conservación del producto y preserven sus condiciones de calidad e inocuidad. “Presentaciones más pequeñas y, sobre todo, que conserven mejor el producto, que no tenga contaminaciones, así puede durar mucho más en el tiempo y se preserva, sobre todo, la calidad del grano”, explicó. La apuesta contempla formatos de 500 gramos, 750 gramos y cinco kilos, con un mayor énfasis en presentaciones de hasta 10 kilos. Actualmente, el arroz embolsado en formatos pequeños representa alrededor del 25% de las ventas de la compañía. La nueva etapa también contempla una inversión en tecnología para el proceso y empaque. ¿Cuándo estarán en el mercado estas innovaciones? Padilla adelantó que estas nuevas presentaciones llegarían al mercado hacia finales de año. “Ya tenemos instalada nuestra planta de proceso”, comentó. Para este desarrollo, la empresa está destinando alrededor de US$ 1.5 millones, inversión que estará enfocada en la incorporación de nueva tecnología. “Estamos invirtiendo en tecnología para llevar al mercado un arroz con mejor fibra y mejores componentes, además de desarrollar presentaciones más pequeñas”, manifestó. La diversificación de Productos Faraón no se limita al arroz. La compañía también participa en la categoría de menestras, donde comercializa lentejas, pallares, garbanzos, arvejas y distintas variedades de frijoles. “Trabajamos tanto con productos nacionales como importados”, alegó. En esta categoría, la compañía también prepara nuevas presentaciones, con una apuesta por formatos pequeños, que estarían disponibles hacia finales de este año. La estrategia de diversificación también contempla ampliar el portafolio de Faraón hacia otras categorías de alimentos de consumo masivo. Entre las categorías que la compañía analiza se encuentran las harinas especiales, como la harina de arroz, además de pastas y aceites, aunque estas incorporaciones todavía se encuentran en proceso de evaluación. El ingreso a estas nuevas categorías está previsto para 2027, con una expectativa de lanzamiento durante el primer semestre de ese año. “La decisión responde a la búsqueda de nuevas oportunidades dentro del consumo masivo y a la demanda de los consumidores, por lo que siempre estamos buscando alternativas de negocios de consumo masivo”, anotó. Una de las principales preocupaciones para la empresa está relacionada con el impacto de Fenómeno El Niño en la producción de los agricultores que la abastecen. En Lambayeque, en particular, Padilla señaló que uno de los principales riesgos asociados a este evento climático es la aparición de plagas como la sogata y la hoja blanca. Ante a este escenario, la empresa viene tomando previsiones para asegurar el abastecimiento y atender la demanda. “Sí estamos previniendo y, en caso de los volúmenes, estamos tratando de tener más producto en stock para sostener la demanda de nuestro mercado”, adelantó. La compañía trabaja con una red de más de 1,000 agricultores y se abastece de distintas zonas de la costa y la selva. Entre ellas se encuentran Lambayeque, Sullana y Piura, además de Tumbes y el valle de Jequetepeque. También obtiene parte de su materia prima de Jaén y Bagua, así como de Nueva Cajamarca, en el Alto Mayo. “Hemos hecho un trabajo interesante con ellos, campaña a campaña, que nos apoyamos mutuamente”, anotó. Esta relación también permite a la empresa anticiparse a eventuales dificultades en la producción. “Si les va mal a ellos, también a nosotros nos va mal”, sostuvo. Actualmente, Productos Faraón concentra su infraestructura industrial en el norte: específicamente su planta está ubicada en Lambayeque (cerca a Chiclayo) y cuenta con un área total de aproximadamente 300,000 metros cuadrados (m2) destinada, entre otros usos, al almacenamiento de arroz. De este espacio, alrededor de 80,000 m2 corresponden al área industrial. La compañía, además, prepara la puesta en operación de una nueva planta en la selva, que complementará las operaciones del norte. “La nueva planta estará en funcionando el próximo año, posiblemente a fines de año”, reveló Padilla. La nueva infraestructura funcionará de manera independiente a la planta del norte y tendrá como uno de sus objetivos acercar a la compañía a los agricultores de esa zona. “Va a complementar la planta del norte, pero independiente, para estar más cerca del agricultor”, expresó. Con esta ampliación, Faraón prevé contar con dos plantas operativas hacia finales de 2027. El ejecutivo precisó que todavía no cuentan con el monto de inversión definido para la nueva planta, que incorporará nueva tecnología.</t>
+          <t>La llegada del Sumo Pontífice es motivo de inmensa alegría para el pueblo peruano, que lo espera con anhelo pues representa el testimonio de especial afecto y cercanía espiritual que el Santo Padre guarda por el Perú, país que también es el suyo.
+El Vaticano anuncia programa oficial de visita de papa León XIV al Perú https://t.co/pVggQUuuib pic.twitter.com/byjGAxnCSs — Agencia Andina (@Agencia_Andina) September 21, 2026 El itinerario oficial incluye las ciudades de Lima, Chiclayo (Lambayeque), Santa Cruz de Succhabamba (Cajamarca), Pucallpa (Ucayali) y Cusco ; y, traza un peregrinaje por la diversidad geográfica, cultural y social del Perú.
+Asimismo, incluye lugares de especial significado para el Santo Padre, donde podrá conectar con el pueblo peruano de la Costa, la Sierra y la Selva de nuestro país, llevando un mensaje de paz, diálogo y reconciliación.
+???????? El Gobierno del Perú recibe con inmenso júbilo y emoción el anuncio oficial de la Santa Sede del programa de la Visita Apostólica de Su Santidad el Papa León XIV, que se llevará a cabo del 11 al 16 de noviembre.
+La tan anhelada llegada del Santo Padre al Perú, testimonio… — Presidencia del Perú ???? (@presidenciaperu) September 21, 2026 Programa oficial de visita de León XIV al Perú: el país espera con júbilo y esperanza la llegada del papa peruano El Perú entero abre sus brazos para recibir al Santo Padre en un encuentro que quedará grabado para siempre en la memoria y el corazón de nuestra nación.
+Más en Andina ???? El papa León XIV se dirige a la multitud desde la ventana del palacio apostólico con vistas a la Plaza de San Pedro durante el rezo del Ángelus dominical en el Vaticano, el 20 de septiembre de 2026.
+https://t.co/FGz2ph5Oro Foto de Andreas SOLARO / AFP pic.twitter.com/NZjYCuglSq — Agencia Andina (@Agencia_Andina) September 20, 2026</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://gestion.pe/economia/empresas/productos-faraon-ventas-crecen-8-y-prepara-nueva-planta-en-la-selva-para-2027-noticia/</t>
+          <t>https://andina.pe/agencia/noticia-peru-se-prepara-para-recibir-jubilo-al-papa-leon-xiv-1092593.aspx</t>
         </is>
       </c>
     </row>
@@ -732,48 +732,630 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>El Comercio</t>
+          <t>Andina</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46280</v>
+        <v>46285</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Papa León XIV: autoridades aceleran preparativos para misa multitudinaria en Pimentel</t>
+          <t>Día del Turismo: manifestaciones culturales que son atractivos turísticos icónicos de Perú</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Las autoridades religiosas, civiles y políticas aceleran los preparativos para la misa multitudinaria que ofrecerá el papa León XIV el próximo 13 de noviembre en las Pampas de Pimentel, en Lambayeque, como parte de su visita al Perú. La organización contempla el acondicionamiento del lugar y la implementación de medidas para recibir a miles de fieles procedentes de distintas regiones del país. El obispo de la Diócesis de Chiclayo, monseñor Edinson Farfán Córdova, informó que ya se inició la planificación de las rutas de acceso y de las actividades previas a la celebración. Estas labores buscan preparar el escenario donde se congregarán los asistentes durante la misa. Según explicó el religioso, existe un cronograma de trabajo con metas a corto, mediano y largo plazo. Entre las principales tareas figuran garantizar los accesos, acondicionar las Pampas de Pimentel y establecer planes de contingencia. “Esta es una fiesta para todo el Perú”, enfatizó Farfán Córdova, quien destacó el trabajo conjunto entre las autoridades y los distintos sectores involucrados en la organización de la celebración. El obispo reconoció que el tiempo constituye uno de los principales desafíos de cara al arribo del papa León XIV. No obstante, señaló que existe disposición para avanzar de manera coordinada y cumplir progresivamente con las tareas previstas. Asimismo, indicó que las decisiones y acciones deberán desarrollarse con transparencia, mediante reuniones permanentes y diálogo entre las instituciones participantes. La misa del 13 de noviembre reunirá en Pimentel a fieles de distintas partes del país.</t>
+          <t>El calendario jubilar peruano es, muy probablemente, el más vasto y variado del mundo.
+Los 365 días del año se celebran diversas festividades de índole costumbrista y religioso en los que aflora un crisol de culturas y creencias que se amalgaman en un rico mestizaje y alcanzan un nivel de cohesión social que identifica a cada comunidad que habita el vasto territorio peruano.
+Según el Directorio Nacional de Festividades el Instituto Nacional de Estadística e Informática (INEI), al año se celebran en Perú más de 6,800 festividades y manifestaciones culturales.
+Algunas de ellas como la Fiesta de las Cruces o del Señor de los Milagros tienen una duración de 31 días , siendo las de mayor duración.
+A nivel de departamentos, Lima, Áncash y Ayacucho concentran el 30% de las festividades del Perú y agosto es el mes con mayor número de festividades con más de 1,000 celebraciones, según el INEI.
+Celebraciones emblemáticas como el Inti Raymi o Fiesta del Sol, los carnavales , la festividad en honor de la Virgen de la Candelaria , la Semana Santa , la Fiesta de San Juan , por citar algunas, generan gran movilización de turistas nacionales y foráneos que muchas veces retornan para volver a vivir una mágica experiencia en Perú.
+En cada festividad regional peruana se exhibe una amplia gama de danzas y música de gran originalidad, alegría y colorido, interpretadas y protagonizadas generalmente por agrupaciones llamadas "comparsas", las cuales identifican a los pueblos y algunas de las cuales han merecido la distinción de Patrimonio de la Humanidad como la Danza de Tijeras, la Huaconada de Mito, la Danza del Wititi, Los Negritos , entre otros.
+Lea también: [ conoce y aprecia las artesanías más emblemáticas de Perú ] País de notables artesanos Todos los turistas que visitan el Perú quedan maravillados con su incontable patrimonio cultural expresado en sus artesanías que enamoran por sus originales diseños, colorido, materiales, creatividad y variedad.
+Textiles, cerámica, orfebrería, talabartería (artesanía en cuero), cerería (artesanía en cera), imaginería, pintura, bisutería , entre otras líneas artesanales que, según la región donde se produzcan, alcanzan un nivel de belleza y excelencia en la elaboración que evidencia el talento los artesanos y artesanas peruanos herederos de una tradición ancestral, enriquecida con el mestizaje y transmitida de generación en generación.
+Ayacucho, Amazonas, Arequipa, Cajamarca, Cusco, Junín, Lambayeque, Loreto, La Libertad, Piura, Puno, San Martín, Ucayali, son los departamentos más emblemáticos en la producción artesanal peruana y cuyas producciones son apreciadas internacionalmente convirtiéndose en un poderoso atractivo para los turistas que llegan al Perú.
+Lea también: [ Día Mundial del Turismo: viaja y admira la vasta herencia histórica y cultural de Perú ] Destino ideal para el turismo vivencial El anhelo de los viajeros que llegan a Perú para conocer su diversidad cultural resulta ampliamente superado en sus expectativas cuando conocen la amplia oferta de lugares donde pueden tener una experiencia inmersiva compartiendo las costumbres y tradiciones de las comunidades que habitan sobre todo en ámbitos rurales de la costa, sierra y selva peruana.
+Y entre amplia oferta de lugares ideales para el turismo vivencial destacan algunos que han sido reconocidos como Pueblos con encanto , gracias a que reúnen atributos culturales y naturales de carácter auténtico y singular con valor simbólico, histórico y turístico que, a través del tiempo, conservan y mantienen viva su identidad, tradiciones y costumbres.
+Estos atributos generan una experiencia turística significativa y memorable en el visitante, siendo el encanto de la población anfitriona y sus expresiones culturales la esencia y el alma del pueblo.
+Los lugares que cuentan actualmente con el reconocimiento de Pueblos con encanto son Ollantaytambo , situado en la provincia cusqueña de Urubamba; los distritos de Yanque y Sibayo , en la provincia arequipeña de Caylloma; Lamas , en el departamento de San Martín; Malabrigo , en la provincia de Trujillo, departamento de La Libertad; Sarhua , distrito de la provincia ayacuchana de Víctor Fajardo; el distrito de Villa Rica , en la provincia de Oxapampa, departamento de Pasco; el distrito de Quinua , en la provincia de Huamanga, departamento de Ayacucho; y el distrito de Chacas , en la provincia de Asunción, departamento de Áncash.
+Lea también: [ Mes del Turismo: ¿Qué atractivos emblemáticos de Arequipa definen su identidad? ] Tierra mística El aura mística que irradia el Perú también es un poderoso imán para el turismo.
+Son muchos los visitantes de todo el planeta que viajan al Perú para conocer lugares con tradición mística , sobre todo en los Andes y la Amazonía, y participan en rituales protagonizados por chamanes o sacerdotes indígenas y mestizos que invocan a las divinidades tutelares o espíritus que viven en montañas, ríos, lagos, lagunas, en la propia tierra como la Pachamama o en el firmamento como el sol, la luna, las estrellas y otros cuerpos celestes.
+Esta experiencia de índole espiritual seduce a los turistas foráneos, quienes valoran el componente cultural expresado en ceremonias en las que se manifiestan la lengua quechua, aimara o amazónica en la que se expresan los chamanes, los elementos de la naturaleza que utilizan en sus rituales (hojas de coca y otras plantas; alimentos como granos, cereales y tubérculos), así como tejidos, prendas de vestir y objetos diversos con simbología religiosa, constituyen el ambiente idóneo para una ritualidad y misticismo únicos.
+Y junto con los rituales es importante destacar los lugares donde se afirma que existen conexiones no solo de índole místico sino también astrológico.
+Entre estos destacan los bosques de piedras de Marcahuasi , en la provincia limeña de Huarochirí; Huayllay en la provincia de Pasco; Pampachiri en la región Apurímac, entre otros que son conocidos por visitantes y lugareños que sostienen que en estos espacios existe una energía especial y que se puede tener contacto con seres de otros planetas.
+Lo que sí es seguro que es que son lugares donde se aprecia a simple vista formaciones rocosas de formas caprichosas gracias a la acción del viento y la lluvia como rostros humanos, cuerpos de animales, figuras geométricas como conos, prismas, pirámides y otros, así como contemplar las diversas constelaciones durante la absoluta oscuridad y silencio de la noche, convirtiéndolos por excelencia en observatorios estelares a campo abierto.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://elcomercio.pe/peru/lambayeque/papa-leon-xiv-autoridades-aceleran-preparativos-para-misa-multitudinaria-en-pimentel-ultimas-noticia/</t>
+          <t>https://andina.pe/agencia/noticia-dia-del-turismo-manifestaciones-culturales-son-atractivos-turisticos-iconicos-peru-1092211.aspx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>El Niño: Minsa prepara a más de 100 profesionales de la salud del norte frente al dengue</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>A través de la Dirección General de Intervenciones Estratégicas en Salud Pública (Dgiesp), equipos especializados del Minsa se desplazaron simultáneamente a estas cuatro regiones para capacitar a médicos y profesionales de enfermería en la detección temprana de signos de alarma, toma de decisiones clínicas, referencia oportuna y manejo adecuado de pacientes con dengue.
+La capacitación incluyó simulaciones de deterioro clínico, diagnóstico diferencial entre dengue y leptospirosis, manejo de pacientes con comorbilidades, organización del triaje, entrenamiento en establecimientos de salud y uso de Telesalud.
+Prepararnos antes para proteger vidas En representación del ministro de Salud, Luis Dyer Fernández, la viceministra de Salud Pública, María Cuba Fuentes, clausuró la jornada y destacó que el objetivo es fortalecer anticipadamente la capacidad de respuesta de los servicios de salud.
+“ Hemos decidido anticiparnos.
+El Minsa está dando un paso adelante, preparando desde ahora a nuestros profesionales de la salud para responder oportunamente ante un posible incremento de casos de dengue.
+Queremos reconocer tempranamente los signos de alarma, actuar antes de que el paciente se agrave y evitar muertes prevenibles.
+Esta preparación comienza en las regiones del norte y avanzará progresivamente para fortalecer nuestra capacidad de respuesta” , señaló la viceministra de Salud Pública, María Cuba Fuentes.
+Los profesionales capacitados tendrán, además, la misión de replicar los conocimientos adquiridos en sus establecimientos y regiones, permitiendo ampliar las capacidades del personal de salud para responder oportunamente frente al dengue.
+Estrategia continuará ampliándose La intervención desarrollada en Tumbes, Piura, Lambayeque y La Libertad constituye un primer paso para la conformación progresiva de la Red Nacional de Referentes Clínicos de Dengue, iniciativa que busca fortalecer la respuesta clínica descentralizada y extender estas capacidades de manera progresiva a otras regiones del país.
+De esta manera, el Minsa avanza en la preparación del sistema de salud frente al dengue, priorizando inicialmente las regiones del norte y fortaleciendo las capacidades del personal para detectar oportunamente los casos de riesgo, brindar una atención adecuada y prevenir complicaciones y muertes.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-el-nino-minsa-prepara-a-mas-100-profesionales-de-salud-del-norte-frente-al-dengue-1092494.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>46284</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>¿Qué dice la historia sobre el impacto del fenómeno El Niño en el Perú?</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Cronistas españoles Desde el punto de vista historiográfico, el cronista español que brindó más referencias sobre la historia temprana del fenómeno El Niño en el Perú es Antonio de la Calancha (1584-1654) , quien en su obra “ Crónica Moralizada de la Orden de San Agustín en el Perú (1638) ” describió las lluvias catastróficas ocurridas en Trujillo, Lambayeque, Zaña y otras localidades de la costa norte peruana.
+Relató el gran evento de lluvias de 1578, considerado por numerosos investigadores como uno de los primeros mega Niño documentados históricamente, que causó inundaciones severas que destruyeron caminos, viviendas, sembríos y sistemas de riego.
+Según Antonio de la Calancha, los ríos se desbordaron, los campos quedaron anegados, se perdieron cosechas, se interrumpieron las comunicaciones por vía terrestre y las lluvias duraron semanas.
+Otro cronista español, José de Acosta (1540-1600) , cuya obra principal “ Historia Natural y Moral de las Indias (1590)”, describió que la costa peruana era normalmente árida y prácticamente sin lluvias, pero registró episodios excepcionales en los que ocurrían precipitaciones inusuales y devastadoras, y documentó impactos sobre la agricultura y la población.
+También observó alteraciones en las corrientes marinas y diferencias térmicas del océano frente a las costas sudamericanas.
+Los climatólogos consideran que sus observaciones constituyen algunas de las primeras descripciones científicas de anomalías océano-atmosféricas compatibles con eventos El Niño.
+Por su parte, el cronista Bernabé Cobo (1582-1657) , en su obra principal “ Historia del Nuevo Mundo” , registró fenómenos naturales extraordinarios observados en el Virreinato del Perú, mencionando la ocurrencia de inundaciones, variaciones climáticas, alteraciones en la producción agrícola y eventos hidrológicos excepcionales.
+Finalmente, el cronista Antonio Vázquez de Espinosa (1570-1630) , en su obra “ Compendio y descripción de las Indias Occidentales” , documentó crecidas de ríos, inundaciones, pérdidas agrícolas, cambios ambientales en la costa peruana y transformaciones temporales del paisaje costero.
+Sus descripciones complementan los de su colega Antonio de la Calancha y permiten conocer eventos climáticos extremos en los siglos XVI y XVII.
+Los documentos legados por estos cronistas constituyen una importante evidencia documental que permite reconstruir la ocurrencia de grandes eventos El Niño varios siglos antes de que existieran estaciones meteorológicas o registros científicos modernos.
+Lea también: [ El Niño Costero: conoce peligros naturales asociados a este fenómeno en el Perú ] Historiadores e investigadores peruanos de los siglos XX y XXI En el siglo XX hubo historiadores e investigadores peruanos que contribuyeron a comprender el fenómeno El Niño y su impacto en el desarrollo de las sociedades desde la época prehispánica.
+Entre ellos mencionamos los siguientes: Lorenzo Huertas Vallejos (1938-2021) , considerado el principal historiador peruano especializado en la historia de El Niño.
+Fue uno de los primeros historiadores peruanos en elaborar cronologías históricas de El Niño desde la época colonial.
+A través de sus obras “Ecología e Historia”, “Historia de los desastres en el Perú”, “Inundaciones y sequías en la historia del Perú”, “Estudios sobre el mega Niño de 1578”, Huertas investigó archivos coloniales, documentos notariales y crónicas españolas para reconstruir eventos climáticos ocurridos entre los siglos XVI y XIX.
+Demostró que las lluvias extraordinarias registradas por los cronistas correspondían a eventos El Niño, que existió una recurrencia histórica de inundaciones en la costa norte, y que los fenómenos climáticos modificaron economías regionales completas.
+María Rostworowski (1915-2016) , es probablemente la historiadora peruana que más influyó en la comprensión de la relación entre clima, recursos marinos y organización social en la costa peruana.
+En sus obras “Recursos naturales renovables y pesca, siglos XVI y XVII”, y “Costa peruana prehispánica”, Rostworowski estudió cómo las sociedades costeñas dependían de los recursos marinos y cómo las alteraciones oceánicas afectaban la economía y la alimentación.
+Sus investigaciones mostraron que los antiguos peruanos conocían períodos de anomalías climáticas; las culturas costeñas desarrollaron estrategias para enfrentar cambios ambientales; las variaciones del mar influyeron en la pesca y el comercio.
+Rostworowski planteó que muchas innovaciones hidráulicas prehispánicas surgieron como respuesta a fenómenos climáticos extremos recurrentes.
+Federico Kauffmann Doig (1928) , en sus obras: “Historia y Arte del Perú Antiguo”, Kauffmann estudió el colapso de determinadas culturas costeñas, la influencia de sequías e inundaciones, los cambios ambientales en la costa norte.
+Propuso que fenómenos climáticos extraordinarios contribuyeron a procesos de crisis en culturas como Moche y Lambayeque .
+Ruth Shady Solís (1946) , antropóloga, arqueóloga, educadora y la más importante investigadora de la civilización Caral, autora del libro “ Caral: la primera civilización de América”, sostiene que en esa sociedad surgida hace 5,000 años y en los poblados que recibieron su influencia, como Vichama, Áspero y Peñico , se afrontaron las consecuencias del cambio climático y del fenómeno El Niño.
+Shady Solís afirma que los estudios y hallazgos efectuados en esos lugares, así como en la Ciudad Sagrada de Caral, dan cuenta de cómo estas poblaciones afrontaron las consecuencias de fenómenos como los de El Niño y el cambio climático, al tener estos un carácter cíclico.
+Agrega que esta cultura recogió información basada en el movimiento de los astros para poder precisar en cuánto tiempo se presentan estas modificaciones que alteraron tanto el modo de vivir de la gente.
+Refiere que en los objetos recientemente hallados en Peñico se muestran rasgos que dan cuenta de fenómenos como inundaciones y carencia de lluvias; incluso graficando el fallecimiento de personas.
+La intención de consignar en objetos esta información habría tenido el objetivo de que la población no olvidara los efectos del cambio climático.
+Esta situación, según las representaciones encontradas en los objetos hallados, se habría debido a la escasez de alimentos generada por la sequía derivada de la falta de lluvias.
+“ En Caral tuvieron que abandonar los centros urbanos porque no tenían agua de los ríos y, por ende, no podían tener alimentación a través de la agricultura ”, subraya la arqueóloga.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-que-dice-historia-sobre-impacto-del-fenomeno-nino-el-peru-1092331.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Temblor en Perú hoy: monitoreo activo por sismo de magnitud 4.0 en Lambayeque</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>El movimiento telúrico ocurrió a las 14:32 horas locales, con una profundidad de 38 kilómetros, y su epicentro fue localizado a 97 kilómetros al oeste del distrito de Pimentel, en la provincia de Chiclayo.
+Según el reporte IGP/Censis, el evento tuvo una latitud -7.11 y longitud -80.77.
+Hasta el momento, las autoridades locales no han reportado daños personales ni materiales por el temblor.
+El evento forma parte de la actividad sísmica monitoreada de forma permanente por el IGP mediante la red sísmica nacional.
+El organismo científico recuerda que el Perú tiene una elevada actividad sísmica debido, principalmente, al proceso de subducción de la placa de Nazca debajo de la placa Sudamericana.
+Una vez más se pone en agenda la importancia de fortalecer la cultura de prevención y la preparación ante emergencias.
+Más en Andina: ?? El @MinamPeru presenta 70 emprendimientos e iniciativas sostenibles en Expoamazónica en Pucallpa https://t.co/GMXYSpnWa3 pic.twitter.com/7SD1hSw7QT — Agencia Andina (@Agencia_Andina) September 18, 2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-temblor-peru-hoy-monitoreo-activo-sismo-magnitud-40-lambayeque-1092394.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Inversión en infraestructura de transporte concesionada sumó US$ 895 millones a agosto</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Las inversiones valorizadas en aeropuertos ascendieron a 484.7 millones de dólares, lo que significó un crecimiento de 53.6% en comparación con el mismo periodo del año anterior.
+ONP y AFP: ¿qué pasará con los aportes si un afiliado cambia de sistema previsional? Por su parte, las inversiones valorizadas en carreteras alcanzaron los 94 millones de dólares, cifra que superó en 188.5% a la registrada entre enero y agosto de 2025.
+En tanto, la concesión de la Línea 2 del Metro de Lima y Callao registró el mayor volumen de inversión acumulada durante el año, con 303.3 millones de dólares valorizados entre enero y agosto, monto superior en 2% al alcanzado en igual periodo de 2025.
+Inversiones valorizadas en agosto Solo en agosto de 2026, las inversiones valorizadas en las infraestructuras de transporte concesionadas sumaron 69.9 millones de dólares.
+En el sector aeroportuario, las inversiones valorizadas ascendieron a 49 millones de dólares.
+De ese total, Lima Airport Partners (LAP) concentró 47.4 millones en inversiones directas en mejoras por el proyecto de ampliación del aeropuerto Jorge Chávez.
+A su vez, el Primer Grupo de Aeropuertos registró valorizaciones por 1.59 millones, vinculadas principalmente al mantenimiento periódico al sistema eléctrico de los aeropuertos de Chiclayo, Piura, Talara y Tumbes.
+En la Red Vial se dinamizaron 13.2 millones de dólares.
+IIRSA Sur Tramo 4 registró inversiones valorizadas por 5.68 millones, destinadas principalmente en el avance de la ejecución de la obra accesoria por seguridad vial-mejoramiento del Sub-Tramo Asillo-San Antón y la ejecución de la obra accesoria inserción urbana y acondicionamiento de drenaje del Centro Poblado de Sangari.
+Asimismo, la concesión IIRSA Norte ejecutó inversiones valorizadas por 3.59 millones en el avance de obras accesorias.
+Por su parte, Autopista del Sol reportó inversiones valorizadas en 1.83 millones, asociadas al avance de la ejecución de las obras obligatorias Evitamiento Chiclayo Zona Norte, Puente Lambayeque e Intercambio Vial Lambayeque, así como de las obras de rehabilitación para la reconstrucción de los sectores afectados por el FEN 2023 en el tramo Trujillo-Chiclayo.
+De igual manera, la concesión Red Vial N.° 6 alcanzó inversiones valorizadas en 1.35 millones en el avance de la obra paso peatonal San Clemente.
+En la Línea 2 del Metro se valorizaron inversiones por 5.15 millones en equipamiento electromecánico, avances de la instalación de las puertas de andén y del sistema de control de pasajeros de las estaciones.
+En el ámbito portuario, la mayor valorización correspondió al Terminal Portuario de Paita, que ejecutó inversiones por 1.87 millones destinadas al sistema de contención de derrumbes del área colindante al terminal portuario y la ampliación de reefer racks.
+Avance de las inversiones Al 31 de agosto de 2026, la inversión valorizada acumulada en las infraestructuras de transporte concesionadas ascendió a 14,820.2 millones de dólares, cifra que representa un avance de 64.6% respecto al compromiso de inversión, que asciende a 22,944.7 millones.
+Más en Andina: La Superintendencia de Banca, Seguros y AFP ( @SBSPERU ) aprobó el Reglamento para la administración del riesgo de sobreendeudamiento de los socios deudores minoristas de las cooperativas de ahorro y crédito no autorizadas a captar recursos del público (Coopac).… pic.twitter.com/tdeeZApUpq — Agencia Andina (@Agencia_Andina) September 18, 2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-inversion-infraestructura-transporte-concesionada-sumo-895-millones-a-agosto-1092376.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Gobernadores regionales emiten pronunciamiento sobre presupuesto 2027</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>En ese sentido, plantearon la necesidad de revisar su asignación para garantizar la continuidad de proyectos y la capacidad de respuesta de las nuevas autoridades.
+De acuerdo con el proyecto presupuestal para el año 2027, los gobiernos regionales son el único nivel de gobierno afectado por un recorte en su Presupuesto Institucional de Apertura (PIA) de inversiones , sufriendo una reducción del 19.12 % .
+“Nos preocupa que los gobiernos regionales enfrenten una reducción cercana al 20 % de su presupuesto de inversión, pese al alto nivel de ejecución que vienen demostrando en sus proyectos y obras”, señaló el titular de la ANGR, Luis Neyra.
+De igual modo, precisó que los gobiernos regionales mantuvieron de manera constante una eficiencia de ejecución presupuestal por encima del 90 % en los últimos años.
+Asimismo, refirió que esta reducción dejará a las nuevas autoridades regionales sin la capacidad financiera requerida para responder a la población, provocando la paralización de proyectos estratégicos destrabados, además de debilitar la gestión de riesgo ante la inminente llegada del fenómeno El Niño (FEN) .
+En el encuentro participaron junto al titular del Consejo de Ministros, Luis Galarreta ; el ministro de Economía y Finanzas, Elmer Cuba ; el viceministro de Hacienda, Erick Lahura ; el viceministro de Desarrollo de Agricultura Familiar e Infraestructura Agraria y Riego, José Tangherlini ; y el viceministro de Gobernanza Territorial, Enrique Vásquez.
+Las autoridades regionales que participaron corresponden a las regiones de Piura, Ayacucho, Lima, Huánuco, Huancavelica, Moquegua, Lambayeque, Pasco, Tumbes, Loreto, Callao, Cajamarca, Amazonas, La Libertad y Áncash.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-gobernadores-regionales-emiten-pronunciamiento-sobre-presupuesto-2027-1092415.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Más de 11 mil casos de violencia escolar en lo que va del 2026: cifras por tipo y región</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ante la denuncia de un presunto abuso sexual contra un estudiante del Liceo Naval Almirante Guise, presuntamente cometido por un grupo de 10 escolares, vuelve a ponerse bajo la lupa la violencia que puede presentarse en los espacios educativos, donde niñas, niños y adolescentes deberían desarrollarse en un entorno seguro y de respeto.
+Lee también: Caso liceo naval: hoy vence plazo de retención en comisaría de escolares denunciados Los reportes del Minedu muestran que el colegio puede convertirse en un escenario de distintas formas de violencia.
+Entre el 1 de enero y el 31 de agosto del 2026, la plataforma SíseVe registró 11 805 reportes de violencia escolar a nivel nacional, que incluyen agresiones entre estudiantes y situaciones en las que estaría involucrado personal de las instituciones educativas.
+Del total de reportes, 5 187 corresponden a violencia física, 4 559 a violencia psicológica y 2 059 a violencia sexual.
+Estas cifras muestran la dimensión de la violencia en el ámbito escolar y evidencian que las agresiones sexuales también forman parte de los casos reportados ante el Minedu.
+A nivel regional A nivel regional, Lima Metropolitana concentra la mayor cantidad de reportes de violencia escolar, con 4 072 casos registrados entre enero y agosto de 2026.
+Le siguen Arequipa, Piura, Junín, Áncash y La Libertad, mientras que Madre de Dios, Huancavelica y Apurímac presentan las cifras más bajas del periodo.
+A continuación, el detalle por región: Lima Metropolitana: 4 072 Arequipa: 730 Piura: 683 Junín: 552 Áncash: 540 La Libertad: 530 Lambayeque: 490 Ica: 414 Cusco: 411 Callao: 423 Lima Provincia: 379 Huánuco: 353 Tacna: 354 San Martín: 322 Cajamarca: 246 Ucayali: 200 Amazonas: 199 Ayacucho: 197 Loreto: 123 Puno: 109 Pasco: 100 Tumbes: 102 Moquegua: 97 Apurímac: 67 Huancavelica: 57 Madre de Dios: 55 Clasificación de la violencia escolar Los reportes de SíseVe agrupan las situaciones de violencia escolar en tres categorías a nivel nacional: física, psicológica y sexual.
+La violencia física comprende el castigo físico, las agresiones que ocasionan lesiones o aquellas que no las generan, así como los casos en los que se utilizan armas.
+En tanto, la violencia psicológica incluye acoso escolar, aislamiento, ciberacoso, discriminación, intimidación, trato humillante, agresiones verbales y situaciones con uso de armas.
+Lee también: Primavera en Lima: más de 20 000 flores amarillas adornarán parques y plazas Por su parte, la violencia sexual contempla el acoso sexual, incluido aquel realizado mediante medios tecnológicos; el hostigamiento sexual; los tocamientos de carácter sexual; los actos de connotación sexual o libidinosos; y la violación sexual, incluso cuando se comete mediante medios tecnológicos.
+Violencia Física Castigo físico (816) Con lesiones (1859) Con uso de armas (64) Sin lesiones (2448) Violencia psicológica Acoso escolar (786) Aislamiento (49) Ciber acoso (564) Uso con armas (27) Discriminación (224) Intimidación (420) Trato humillante (1226) Verbal (1263) Violencia sexual Acoso sexual (92) Acoso sexual a través de medios tecnológicos (59) Hostigamiento sexual (213) Tocamientos, actos de connotación sexual o actos libidinosos (1423) Violación sexual (156) Violencia con fines sexuales a través de medios tecnológicos (116) Más en Andina ? El cardenal Carlos Castillo, arzobispo de Lima, anunció que se realizan gestiones para que la imagen del Señor de los Milagros se encuentre con el papa León XIV durante el último día de su visita a Lima.
+https://t.co/lg713AIZrF pic.twitter.com/S0sA4l1Pql — Agencia Andina (@Agencia_Andina) September 18, 2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-mas-11-mil-casos-violencia-escolar-lo-va-del-2026-cifras-tipo-y-region-1092355.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>El Niño Costero: Chiclayo pone a prueba sus sistemas contra inundaciones</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>El ejercicio permitió evaluar las acciones y la articulación ante una eventual emergencia generada por lluvias intensas.
+Así, se verificó el correcto funcionamiento de los SARE El Amauta La Victoria; el hospital Regional, Villareal Yortuque y la urbanización San Lorenzo, que permiten atender a una población expuesta de más de 67,000 habitantes.
+La actividad contó con la participación de la alcaldesa de la provincia de Chiclayo, Janet Cubas; la alcaldesa del distrito de José Leonardo Ortiz, Elvia García; representantes del Gobierno Regional de Lambayeque, funcionarios del Ministerio de Vivienda, Construcción y Saneamiento (MVCS), EPS Epsel, Policía Nacional, Ejército y otras entidades.
+“A mí me complace que ya hayamos logrado el objetivo.
+Veo con muy buenos ojos que hayamos encontrado 11 puntos por mejorar; eso quiere decir que la simulación está funcionando” , indicó el ministro Arnillas.
+Asimismo, animó a los participantes a seguir trabajando, porque el fenómeno El Niño (FEN), según las proyecciones, será de gran intensidad y estos ejercicios servirán para salvar vidas.
+Encauzamiento del río La Leche Como parte de la preparación frente al FEN, el ministro Arnillas supervisó la intervención en el río La Leche, donde se han colocado geobolsas y se ejecutan trabajos destinados a recuperar la capacidad hidráulica del cauce y reducir el riesgo ante el incremento de caudales durante la temporada de lluvias, en beneficio de 4,408 pobladores.
+“El Ministerio de Vivienda tiene 45 puntos de intervención en la región Lambayeque, en los que venimos trabajando desde enero.
+Desde julio a la fecha, hemos intensificado las actividades, trabajando en doble turno y duplicando los turnos de la maquinaria”, indicó.
+Supervisión de infraestructura La jornada también incluyó la supervisión de acciones destinadas a fortalecer el abastecimiento de agua potable.
+Arnillas cumplió con el compromiso que asumió con los pobladores del pueblo joven California de concluir los trabajos de instalación de un pozo tubular, que les permite contar con agua que se distribuye a traves de camiones cisterna para la población.
+También constató los trabajos realizados en la EBAR Ciudad de Dios, en el distrito de San José, con el fin de dar solución al problema de bombeo de aguas residuales para su evacuación mediante canales.
+Con estas acciones, el MVCS fortalece la preparación de Lambayeque frente al FEN, que combinan ejercicios de respuesta ante emergencias con intervenciones preventivas y el mejoramiento de los servicios de agua y saneamiento para reducir los riesgos que podrían afectar a la población.
+Durante 2026, el sector Vivienda ha ejecutado 34 intervenciones en Lambayeque, de las cuales 30 corresponden a trabajos de limpieza y descolmatación en las provincias de Chiclayo, Ferreñafe y Lambayeque.
+Estas acciones permitieron retirar más de 182,000 m³ de material sedimentado, equivalente a 12,165 volquetadas, en una longitud de 62.1 km de cauces, en beneficio de cerca de 64,000 pobladores.
+Sectores críticos La alcaldesa Cubas, por su parte, señaló que el SARE de La Videnita se encuentra operativo y que las mangas instaladas alcanzan cerca de 700 metros.
+Sin embargo, advirtió que existen sectores críticos ubicados a tres o cuatro kilómetros de estos sistemas, donde sería necesario contar con camiones cisterna para evacuar rápidamente el agua acumulada.
+La autoridad municipal también planteó evaluar la construcción de cámaras de bombeo para superar las limitaciones de distancia, al recordar que una motobomba puede impulsar el agua mediante sus mangas entre 500 y 570 metros.
+Entre los sectores identificados como de mayor atención figuran la vía de evitamiento y el pueblo joven 4 de Noviembre, donde se requieren medidas adicionales para responder ante una eventual emergencia por lluvias intensas.
+Más en Andina: ?????? Virgilio Martínez recibió el Andorra Taste Award 2026 por su trabajo en favor de la biodiversidad peruana y una propuesta que conecta territorio, productos nativos, conocimientos ancestrales y comunidades.
+?? https://t.co/IBTubyPfkP pic.twitter.com/gOe894WSBw — Agencia Andina (@Agencia_Andina) September 19, 2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-el-nino-costero-chiclayo-pone-a-prueba-sus-sistemas-contra-inundaciones-1092421.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>¿Necesitas tramitar o recoger tu DNI? Reniec atenderá este sábado 19 y domingo 20</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>La entidad registral exhorta a los ciudadanos a revisar la lista de sedes, ubicaciones y horarios de atención para programar su visita .
+A continuación, conoce las oficinas de Reniec que abrirán sus puertas al público durante este fin de semana.
+Lee también: Reniec habilita nuevas sedes para trámites de DNI: conoce cómo reservar tu cita vía web Sedes de Reniec que atenderán hoy sábado 19 de setiembre Este sábado 19 de setiembre, Reniec atenderá en varias oficinas ubicadas en Piura, Lambayeque, Tumbes, Cajamarca, La Libertad, Loreto, San Martín, Áncash, Junín, Ayacucho, Arequipa, Moquegua, Madre de Dios y Cusco.
+Además, atenderá en sedes ubicadas en Lima, Puno, Ica, Ayacucho, Ucayali, Huánuco, Huancavelica, Cajamarca y Amazonas.
+El horario de atención será diferenciado.
+En algunas oficinas será de 08.15 a.
+m.
+a 12.45 p.
+m., mientras que en otras de 08.30 a.
+m.
+a 1.00 p.
+m.
+Conoce las ubicación y horarios de atención de oficinas en este ENLACE .
+Sedes de Reniec que atenderán el domingo 20 de Setiembre Este domingo 20 de setiembre, Reniec atenderá en oficinas ubicadas en Piura, Trujillo, Ayacucho y Puno desde las 08:15 a.m.
+hasta las 12.45 p.m., para entregas y trámites de DNI.
+Además, atenderá en la oficina registral de Cusco, en el mismo horario, solo para entregas de DNI.
+Ver ENLACE .
+?? ¡Tramita tu DNI electrónico gratis! Niños y niñas, adultos mayores, personas con discapacidad, personas en situación de pobreza y pobreza extrema, entre otros, pueden obtener su documento nacional de identidad sin costo, según explica la jefa del @ReniecPeru , Carmen Velarde.… pic.twitter.com/nQtGIya7nB — Agencia Andina (@Agencia_Andina) September 18, 2026 Trámites virtuales, pago y recojo de DNI Los ciudadanos también pueden realizar varios trámites de identificación y de registro civil de manera virtual por medio de la página web oficial de Reniec.
+Conoce todos en este ENLACE .
+Lee también: Reniec realizará campaña gratuita para el DNI: conoce horarios, lugares y beneficiarios El pago por trámites lo pueden realizar por medio de Yape, agente BCP, Banco de la Nación o págalo.pe.
+En el caso de Yape, deben generar un ticket de pago a través de este ENLACE , seleccionar el código correspondiente al trámite e ingresar el número de ticket en la aplicación, en la opción Yapear servicios &gt; Reniec para finalizar el pago.
+Los ciudadanos que ya realizaron su trámite ya sea de manera virtual o presencial pueden revisar a través de este ENLACE si su DNI está listo para recojo.
+Si el estado de trámite figura al 100 %, se pueden dirigir a la sede que eligieron para recoger su documento.
+Más en Andina : ?? Caso Liceo Naval: el Poder Judicial dictó medidas de protección para resguardar a la presunta víctima durante las investigaciones.
+Los adolescentes denunciados tienen prohibido utilizar plataformas digitales y redes sociales contra el agraviado y deberán recibir terapias… pic.twitter.com/OSlKDMZTQD — Agencia Andina (@Agencia_Andina) September 18, 2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-necesitas-tramitar-o-recoger-tu-dni-reniec-atendera-este-sabado-19-y-domingo-20-1092300.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Gobernadores regionales tendrán reunión extraordinaria hoy en Lima</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>El evento, al cual se ha invitado a los medios de comunicación, se llevará a cabo a las 16:30 horas en el Colegio Médico del Perú, sito en avenida 28 de Julio, en el distrito de Miraflores.
+Cabe indicar que en el marco de las acciones orientadas a consolidar la gobernabilidad y el trabajo articulado en el país, el presidente del Consejo de Ministros, Luis Galarreta, sostuvo una reunión de trabajo con el consejo directivo de la Asamblea Nacional de Gobiernos Regionales (ANGR), liderado por su presidente y gobernador regional de Piura, Luis Neyra León, y su vicepresidente y gobernador regional de Lambayeque, Jorge Pérez Flores.
+En el encuentro se reafirmó el compromiso del Gobierno Nacional y los gobiernos regionales de impulsar agendas conjuntas en favor del desarrollo territorial.
+Durante la sesión de trabajo, el jefe del Gabinete Ministerial y los líderes de la ANGR abordaron prioridades de interés nacional, entre las que destacan la implementación de medidas ante el fenómeno El Niño, el reforzamiento de la seguridad ciudadana y la aceleración de la ejecución de proyectos de inversión pública.
+En la cita participaron también las representaciones de los gobiernos regionales de Moquegua, Tumbes y Huánuco.
+El encuentro estratégico se llevó a cabo como antesala a la Asamblea Nacional de Gobernadores Regionales , evento que se desarrolla hoy en Lima.
+Más en Andina ??? El Gobierno otorgará un subsidio económico temporal para los conductores de mototaxis (categoría vehicular L5) en los departamentos de Loreto, Ucayali y Madre de Dios, con el objetivo de enfrentar el alza de los precios de los combustibles.
+https://t.co/0E6DIJattb pic.twitter.com/mZ5xRuhoKN — Agencia Andina (@Agencia_Andina) September 18, 2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-gobernadores-regionales-tendran-reunion-extraordinaria-hoy-lima-1092294.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>El Perú conectará con el mundo en la feria Expoalimentaria 2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Las agroexportaciones peruanas (tradicionales y no tradicionales) sumaron 6,567 millones 787,000 dólares entre enero y julio del 2026.
+“Esta cifra refleja un ligero incremento de 2% y evidencia la importancia de seguir impulsando la presencia de estos productos en los principales mercados del mundo”, subrayó Adex.
+Para la Expoalimentaria 2026 se espera la participación de 1,600 compradores nacionales e internacionales, quienes tendrán contacto con alrededor de 735 expositores de distintos países.
+Desde EE.UU.
+llegarán firmas como Walmart, interesada en frutas frescas y semiprocesadas; Valle Fruit, en búsqueda de mango congelado orgánico y convencional; MEGA Brand Development, que demanda bebidas energizantes con extractos naturales; y ALK Fresh, especializada en la adquisición de frutas congeladas.
+Como parte de la delegación de Europa estarán Cotswold Fayre de Reino Unido (snacks de yuca y galletas dulces), Solidar Monde de Francia (pitahaya, jengibre, chía y harina de banano), Confluencia de Italia (palta fuerte, pulpa de mango y concentrados de chicha morada) y Mercontrol de España (salsas preparadas, ajos, ajíes y páprika).
+De América Latina llegarán representantes de El Dorado de Uruguay (conservas de pescado), Colombina de Colombia (ajíes peruanos y pasta de tomate), De Marchi de Brasil (arándanos y espárragos), Mafralac de Argentina (saborizantes), Supermercados Cugat de Chile (chocolates), entre otras.
+En el marco de la Expoalimentaria, ADEX Consulting realizará una Rueda de Negocios, que espera superar las 3,200 citas comerciales.
+La expectativa para la actual edición es lograr un monto mayor a los 905 millones de dólares en transacciones futuras.
+El portafolio exportador de nuestro país destaca por los arándanos, uvas, paltas, mangos, mandarinas, bananas, espárragos, alcachofas, granos andinos, café, cacao, capsicum, jengibre y otros.
+Parte de la oferta de las pequeñas empresas se ubicará en el pabellón Pymexporta.
+A ellas se sumarán compañías proveedoras de envases, empaques, maquinaria y servicios logísticos, con soluciones orientadas a fortalecer la competitividad de toda la cadena.
+El mundo y las regiones presentes Se ha confirmado la asistencia de representantes de empresas expositoras de los cinco continentes, así como la instalación de seis pabellones correspondientes a Argentina, Brasil, Ecuador, Países Bajos, Italia e Indonesia.
+De la misma forma, se mostrarán bienes provenientes de diversas zonas del Perú.
+Adicionalmente, los gobiernos regionales de San Martín, Junín, Cajamarca y Lambayeque contarán con áreas de exhibición para poner en valor lo mejor de su portafolio.
+Temas claves También se llevarán a cabo conferencias magistrales enfocadas en Sostenibilidad y producción responsable, Mercado orgánico global, Mercados y negocios internacionales, Tecnología y foodtech, Logística inteligente y cadenas de suministros, e Innovación.
+Las charlas estarán a cargo de ponentes nacionales y foráneos, como el gerente de Ventas para Latinoamérica de Coface, el colombiano Diego Rincón; desde Reino Unido estará el CEO de Cotswold Fayre, Paul Hargreaves; y de Países Bajos expondrá el Account manager en Eurofins food, feed &amp; water Benelux de Agrorum, Dilara Ersahin.
+Exportaciones Entre enero y julio del 2026 resaltaron en la oferta agro las paltas (1,127 millones 685,000 dólares), uvas frescas (805 millones 942,000 dólares), arándanos (620 millones 240,000 dólares) y café sin descafeinar (477 millones 402,000 dólares).
+Se sumaron los mangos, cacao en grano, espárragos y otros.
+EE.UU.
+(2,050 millones de dólares) y Países Bajos (1,055 millones de dólares) fueron sus principales receptores, acumulando el 47% del total.
+España, Chile y México completaron el top five.
+Los auspiciadores de la Expoalimentaria 2026 son: Talma Servicios Aeroportuarios, Alfosac, Evergreen, Garantía Capital, Coface, Interbank, Universidad de Lima, IIRSA Sur, Chep, Cold Import, Agrorum, Cooperación Alemana para el Desarrollo (implementada por la GIZ y la Unión Europea), Cenfrico, ICE (Agencia Italiana para el Comercio Exterior – Embajada de Italia), United Cargo Company, APM Terminals, Veritrade, Orginor, Reyemsa, Primax Gas y Puerto de Paracas.
+Más en Andina: ?? Arequipa destaca como una región con oportunidades para la inversión y como la segunda economía más importante del interior del país.
+Sus exportaciones pasaron de US$612 millones en 2005 a US$8,466 millones en 2025, impulsadas principalmente por la minería.
+La región… pic.twitter.com/J37LNYB1TV — Agencia Andina (@Agencia_Andina) September 14, 2026</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-el-peru-conectara-con-mundo-la-feria-expoalimentaria-2026-1092287.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Misa del papa León XIV en Pimentel: delimitan áreas para trabajos de acondicionamiento</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>La visita de campo permitió hoy identificar las zonas prioritarias de intervención y establecer las acciones que asumirá el sector empresarial para contribuir a la preparación del espacio que recibirá a miles de fieles durante la visita del santo padre.
+En la jornada participaron representantes de la Cancillería, el Gobierno Regional de Lambayeque, la Municipalidad Distrital de Pimentel, sector empresarial y diversas instituciones, quienes recorrieron el terreno para definir una hoja de ruta concreta y pasar de la planificación a la ejecución.
+El presidente de la Cámara de Comercio y Producción de Lambayeque (CCPL), Juan Manuel Scander Chikhani, reafirmó el compromiso del empresariado regional de sumar esfuerzos para que Pimentel se encuentre en condiciones adecuadas para este acontecimiento de alcance nacional.
+Centro de operaciones Como parte de este compromiso, la CCPL ha puesto a disposición sus instalaciones para el funcionamiento del centro de operaciones destinado a la prensa internacional y la Cancillería, que permitirá facilitar las labores de coordinación y cobertura durante la visita papal.
+Con la delimitación georreferenciada de los espacios y la definición de las primeras intervenciones, Pimentel entra así en una fase decisiva de preparación, en la que el trabajo conjunto entre autoridades y sector privado será clave para acondicionar el escenario de la celebración religiosa.
+Se informó que la Cámara de Comercio continuará acompañando las acciones de articulación institucional para contribuir a que Lambayeque esté preparado para recibir al papa León XIV y a los miles de peregrinos que llegarán a la región.
+Más en Andina: ????? El Gobierno atiende 536 puntos críticos del país como parte de las acciones de preparación frente al fenómeno El Niño 2026-2027.
+El ministro Marco Vinelli informó que la descolmatación del río Piura alcanza un 56% de avance en la zona de Los Ejidos.
+??… pic.twitter.com/0YymH6FkxL — Agencia Andina (@Agencia_Andina) September 19, 2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-misa-del-papa-leon-xiv-pimentel-delimitan-areas-para-trabajos-acondicionamiento-1092434.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46283</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Incautan 100 armas y más de mil kilos de explosivos y pirotécnicos en 13 regiones</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Estas intervenciones se realizaron en Áncash, Apurímac, Arequipa, Cajamarca, Cusco, Ica, Junín, La Libertad, Lambayeque, Loreto, Piura, Puno y Ucayali.
+Estas han permitido verificar las condiciones de seguridad en la tenencia de armas de fuego y prevenir la fabricación, almacenamiento, comercialización y uso de productos pirotécnicos y explosivos sin la autorización correspondiente.
+Como parte de este despliegue, las jefaturas zonales de Sucamec realizaron intervenciones a empresas de seguridad privada, usuarios de armas de fuego y establecimientos vinculados a las actividades de explosivos y productos pirotécnicos.
+Las incautaciones allí realziadas comprendieron 100 armas de fuego y 604 municiones, además de 734 kilos de productos pirotécnicos y 450 kilos de explosivos, informó el Ministerio del Interior.
+“Estamos intensificando la fiscalización en todo el país para detectar situaciones irregulares y evitar que armas, municiones, explosivos o productos pirotécnicos sean utilizados fuera de las condiciones establecidas por ley”, señaló el titular de la Sucamec, Eswin Manay Guerrero.
+[Lea también: Impulsan red de 7 puertos para garantizar abastecimiento de alimentos y ayuda ] El armamento intervenido en las empresas de seguridad presentaba que comprometían las condiciones exigidas para su custodia, entre ellas fallas en los sistemas de videovigilancia y alarmas, así como deficiencias en los registros de control y custodia.
+Asimismo, las fiscalizaciones a usuarios permitieron detectar armas vinculadas a licencias canceladas y vencidas.
+Asimismo, acciones que Sucamec efectuó junto a la Policía Nacional y la Superintendencia Nacional de Aduanas y de Administración Tributaria, permitieron detectar talleres que operaban de manera informal y materiales que eran trasladados clandestinamente.
+En ese contexto, se decomisaron 694 kilos de productos pirotécnicos en Junín y Áncash; además de 40 kilos en Lambayeque , durante una acción a una empresa que los iba a trasladar como encomienda.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-incautan-100-armas-y-mas-mil-kilos-explosivos-y-pirotecnicos-13-regiones-1092369.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Anadarko ratifica su interés en Perú y avanza a la perforación exploratoria en Lote Z-62</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>El ministro de Energía y Minas, Guillermo Shinno, sostuvo una reunión con representantes de Anadarko-Oxy, Pedro Romero, Douglas Roberts y César Ardiles, quienes informaron sobre los avances de sus actividades de exploración en los lotes Z-61, Z-62 y Z-63, ubicados frente a las costas de La Libertad y Lambayeque, y ratificaron la decisión de continuar explorando el potencial de hidrocarburos del norte del país.
+Durante el encuentro, la compañía explicó que viene culminando la interpretación de los estudios de sísmica 2D y 3D, que permitieron identificar prospectos de alto potencial hidrocarburífero, y que las evidencias naturales de hidrocarburos detectadas mediante imágenes satelitales y drop cores respaldan la existencia de un sistema petrolero activo.
+“En base a los resultados obtenidos, Anadarko indicó que ha decidido ingresar a la tercera fase del proyecto, que contempla el compromiso de realizar una perforación de un pozo exploratorio en el Lote Z-62, el cual permitirá contar con mayor información y evaluar futuras oportunidades de desarrollo e inversión en la zona”, enfatizó el Minem.
+El ministro Shinno destacó los avances alcanzados por la compañía y señaló que el Gobierno trabaja para fortalecer la competitividad del país, atraer nuevas inversiones y promover la puesta en valor de sus recursos energéticos.
+En ese sentido, resaltó que la continuidad de estas iniciativas contribuye a generar nuevas oportunidades de desarrollo y crecimiento para el país.
+Agregó que resulta clave contar con una permisología eficiente que otorgue predictibilidad a las inversiones y permita avanzar oportunamente con las iniciativas, respetando las obligaciones ambientales y sociales.
+A su turno, la viceministra de Hidrocarburos, Iris Cárdenas, explicó que el sector viene trabajando en propuestas normativas orientadas a agilizar estos procesos.
+“El Minem reafirma su disposición de fortalecer la coordinación entre las entidades competentes del sector, generando condiciones que acompañen y faciliten nuevas inversiones y contribuyan al fortalecimiento del sector hidrocarburos y de la seguridad energética del país”, puntualizó el ministerio.
+Más en Andina: ?? Arequipa destaca como una región con oportunidades para la inversión y como la segunda economía más importante del interior del país.
+Sus exportaciones pasaron de US$612 millones en 2005 a US$8,466 millones en 2025, impulsadas principalmente por la minería.
+La región… pic.twitter.com/J37LNYB1TV — Agencia Andina (@Agencia_Andina) September 14, 2026</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-anadarko-ratifica-su-interes-peru-y-avanza-a-perforacion-exploratoria-lote-z62-1092263.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Andina</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>46282</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Chiclayo implementa 60 señales turísticas para fortalecer la Ruta del Papa León XIV</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>El subgerente de Turismo y Cultura de la comuna chiclayana, David Cárdenas Angulo, informó en diálogo con la Agencia Andina que el componente de señalización registra un 50 % de avance y que la instalación de las estructuras restantes culminará durante septiembre.
+“En total se implementarán 60 señales turísticas, entre orientativas e interpretativas, ubicadas en puntos estratégicos y principales atractivos de la provincia de Chiclayo y otros espacios vinculados a la Ruta turística del Papa León XIV ”, apuntó.
+Refirió que la señalización interpretativa incluirá paneles con información en español, inglés y sistema braille, con datos históricos, arquitectónicos y turísticos de los atractivos.
+Entre los lugares considerados figuran la Iglesia San Pedro de Monsefú, la Iglesia María Magdalena de Ciudad Eten, el Parque Principal de Chiclayo, el Santuario Nuestra Señora de la Paz y otros puntos de interés.
+Cárdenas, explicó que el diseño responde al Manual de Señalización Turística y contempla una iconografía específica para facilitar la identificación de cada atractivo .
+Asimismo, las propuestas fueron revisadas por especialistas y cuentan con opiniones favorables de las entidades competentes.
+La iniciativa se ejecuta en el marco de un convenio interinstitucional entre el Ministerio de Comercio Exterior y Turismo (Mincetur) y la Municipalidad Provincial de Chiclayo, que contempla acciones de señalización turística, promoción de la inversión privada, promoción turística y formalización.
+La comuna espera que el nuevo sistema permita a los visitantes orientarse con mayor facilidad, conocer la historia y el valor arquitectónico de los lugares vinculados a la Ruta del Papa León XIV y ampliar su recorrido por la provincia.
+De esta manera, Chiclayo busca llegar a noviembre, cuando se prevé la presencia del papa León XIV, con una infraestructura de orientación turística que facilite el desplazamiento de los miles de visitantes nacionales y extranjeros que se movilizarán por los principales atractivos de Lambayeque.
+Más en Andina: ??? Más de 250 mil personas están en riesgo muy alto por deslizamientos asociados a las lluvias en 8 regiones.
+Ayacucho concentra 119,875 pobladores en esta condición, según el Cenepred.
+?? https://t.co/DMad7tei3D pic.twitter.com/BHXjT3CZiG — Agencia Andina (@Agencia_Andina) September 17, 2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://andina.pe/agencia/noticia-chiclayo-implementa-60-senales-turisticas-para-fortalecer-ruta-del-papa-leon-xiv-1092217.aspx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>El Comercio</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B23" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Papa León XIV: autoridades aceleran preparativos para misa multitudinaria en Pimentel</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Las autoridades religiosas, civiles y políticas aceleran los preparativos para la misa multitudinaria que ofrecerá el papa León XIV el próximo 13 de noviembre en las Pampas de Pimentel, en Lambayeque, como parte de su visita al Perú. La organización contempla el acondicionamiento del lugar y la implementación de medidas para recibir a miles de fieles procedentes de distintas regiones del país. El obispo de la Diócesis de Chiclayo, monseñor Edinson Farfán Córdova, informó que ya se inició la planificación de las rutas de acceso y de las actividades previas a la celebración. Estas labores buscan preparar el escenario donde se congregarán los asistentes durante la misa. Según explicó el religioso, existe un cronograma de trabajo con metas a corto, mediano y largo plazo. Entre las principales tareas figuran garantizar los accesos, acondicionar las Pampas de Pimentel y establecer planes de contingencia. “Esta es una fiesta para todo el Perú”, enfatizó Farfán Córdova, quien destacó el trabajo conjunto entre las autoridades y los distintos sectores involucrados en la organización de la celebración. El obispo reconoció que el tiempo constituye uno de los principales desafíos de cara al arribo del papa León XIV. No obstante, señaló que existe disposición para avanzar de manera coordinada y cumplir progresivamente con las tareas previstas. Asimismo, indicó que las decisiones y acciones deberán desarrollarse con transparencia, mediante reuniones permanentes y diálogo entre las instituciones participantes. La misa del 13 de noviembre reunirá en Pimentel a fieles de distintas partes del país.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://elcomercio.pe/peru/lambayeque/papa-leon-xiv-autoridades-aceleran-preparativos-para-misa-multitudinaria-en-pimentel-ultimas-noticia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>El Comercio</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
         <v>46279</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Papa León XIV está de cumpleaños: Chiclayo celebra al sumo Pontífice y prepara su esperado reencuentro</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>El papa León XIV cumple 71 años este lunes 14 de septiembre, una fecha que ha sido recibida con especial emoción en Chiclayo, ciudad donde Robert Prevost desarrolló una importante etapa de su labor pastoral y que hoy lo recuerda como un pastor cercano. La celebración en Lambayeque incluye mensajes de cariño, música y oración, además de una jornada cultural y religiosa organizada por el Gobierno Regional de Lambayeque y la Diócesis de Chiclayo. El homenaje también se produce en medio de la expectativa por la próxima visita del Santo Padre al Perú. Con voces cargadas de emoción, los chiclayanos dedicaron un saludo especial al Santo Padre, acompañado de una canción tradicional que buscó transmitirle el cariño de quienes lo recuerdan desde su etapa como pastor en Lambayeque. “¡Despierta, Papa, despierta, mira que ya amaneció, ya los pajaritos cantan, la luna ya se metió!”, entonaron los participantes antes de cerrar el mensaje con un: “¡Feliz cumpleaños, Papa León!”. Desde la ciudad que considera parte fundamental de su historia pastoral, los fieles, liderados por el obispo de la Diócesis de Chiclayo, monseñor Edinson Farfán, hicieron llegar al pontífice un saludo fraterno a través de las redes sociales. “Gracias por ser un buen pastor y por ser la luz de todos nosotros”, expresaron los participantes, quienes destacaron la vocación de servicio de León XIV y su cercanía durante los años que permaneció en la región. El homenaje estuvo marcado por distintas expresiones de afecto hacia el pontífice. “Orgullosa de ti, de tu labor”, “que Dios siga derramando muchas bendiciones a todos los peruanos” y “te esperamos con mucho amor aquí en tu ciudad, Chiclayo”, fueron algunos de los mensajes dedicados a León XIV. El saludo terminó con una declaración colectiva que refleja el vínculo que la ciudad mantiene con quien fuera su obispo: “¡Feliz cumpleaños desde tu tierra querida, Chiclayo!”. La celebración no solo busca recordar el cumpleaños del Santo Padre, sino también reafirmar el deseo de los fieles de volver a encontrarse con él en la ciudad donde desarrolló parte importante de su trayectoria religiosa. Como parte de las celebraciones, el Gobierno Regional de Lambayeque y la Diócesis de Chiclayo convocaron a la ciudadanía a participar este lunes 14 de septiembre en una jornada cultural y religiosa dedicada al papa León XIV. La actividad se desarrollará desde la 1:30 p. m. en el atrio de la Catedral de Chiclayo, uno de los principales espacios religiosos y culturales del centro histórico de la ciudad. La jornada reunirá expresiones culturales y religiosas y estará abierta a la población local y a los visitantes que quieran sumarse al homenaje por los 71 años del Santo Padre. El encuentro busca expresar el reconocimiento y cariño de los lambayecanos hacia León XIV, así como mantener viva la relación que construyó con la comunidad durante sus años de labor pastoral. El homenaje de Chiclayo se suma al saludo enviado por la Conferencia Episcopal Peruana (CEP) con motivo del cumpleaños del Santo Padre. La institución religiosa expresó sus buenos deseos al pontífice y destacó la importancia de acompañarlo mediante la oración de los fieles peruanos. Su mensaje también estuvo acompañado de un video especial elaborado por la ocasión. “¡Feliz cumpleaños, Papa León XIV! El Perú lo espera con alegría, cariño y oración”, expresó la CEP. El mensaje refleja además la expectativa existente en el país ante la próxima visita del pontífice, especialmente en Chiclayo, donde sus antiguos fieles esperan volver a recibirlo. Más allá del cumpleaños, la celebración tiene un significado especial para Chiclayo. Para sus habitantes, León XIV no es solo el actual sucesor de Pedro, sino también el religioso que durante años compartió con la comunidad local su labor pastoral. Por ello, la Diócesis de Chiclayo y las autoridades regionales han comenzado a preparar el ambiente para la eventual llegada del Santo Padre, mientras los fieles expresan públicamente su deseo de reencontrarse con él. La Conferencia Episcopal Peruana también anunció la apertura de un espacio oficial para acompañar los preparativos de la próxima visita de León XIV al Perú y promover que los católicos vivan espiritualmente la espera. La jornada de celebración por los 71 años del papa León XIV se convierte así en una expresión de cariño de una ciudad que conserva un vínculo especial con el pontífice. Entre música, oraciones y mensajes de afecto, Chiclayo vuelve a pronunciar el nombre de quien fuera su obispo y mira hacia Roma mientras espera el próximo reencuentro. “¡Feliz cumpleaños, Papa León! Un fuerte abrazo desde Chiclayo, la ciudad de la amistad, la tierra del Dios que tanto amas. ¡Te esperamos en Chiclayo!”.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>https://elcomercio.pe/peru/lambayeque/papa-leon-xiv-esta-de-cumpleanos-chiclayo-celebra-al-sumo-pontifice-y-prepara-su-esperado-reencuentro-ultimas-noticia/</t>
         </is>

</xml_diff>